<commit_message>
small chnages on the pcb and extend BOM to PCB assembly parts
</commit_message>
<xml_diff>
--- a/production/PCB/keybowl_bom.xlsx
+++ b/production/PCB/keybowl_bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felix\Desktop\homeassistant_keybowl\production\PCB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65260762-D702-48F4-BC0B-0FADC1C02CC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD2CF2FE-28F8-4B9B-BF69-BACA1C5C9E82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="38700" windowHeight="15885" xr2:uid="{84AA4AA4-4591-4CB7-AD30-DDE362546BAC}"/>
+    <workbookView xWindow="11280" yWindow="21480" windowWidth="29040" windowHeight="16440" xr2:uid="{84AA4AA4-4591-4CB7-AD30-DDE362546BAC}"/>
   </bookViews>
   <sheets>
     <sheet name="keybowl_bom" sheetId="1" r:id="rId1"/>
@@ -97,10 +97,10 @@
     <t>C842287</t>
   </si>
   <si>
-    <t>100uF</t>
-  </si>
-  <si>
-    <t>C23692977</t>
+    <t>10uF</t>
+  </si>
+  <si>
+    <t>C39060</t>
   </si>
 </sst>
 </file>

</xml_diff>